<commit_message>
adding documents from Lana
</commit_message>
<xml_diff>
--- a/Application Status Push Notification - Push Notify usage map 5.1.2026.xlsx
+++ b/Application Status Push Notification - Push Notify usage map 5.1.2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://libertylife-my.sharepoint.com/personal/e97529_atheneusa_com/Documents/Documents/Application Status_App Status Push/Application Status Push Notifications-Share Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{EAD004BD-F2A7-4D3E-8276-48FC41559210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{322A6234-A1AA-45AF-A516-A8E28FD74668}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{EAD004BD-F2A7-4D3E-8276-48FC41559210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12E125D9-79BB-47A7-BCB5-1BFF91A49B20}"/>
   <bookViews>
-    <workbookView xWindow="5616" yWindow="3504" windowWidth="17280" windowHeight="9960" xr2:uid="{9F51EC60-E570-4BE0-850C-6F12511B0CE1}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{9F51EC60-E570-4BE0-850C-6F12511B0CE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Dictionary Use Case Map" sheetId="2" r:id="rId1"/>
@@ -781,9 +781,6 @@
     <t>Best Practice is to provide as much detail as is available to resolve issue.</t>
   </si>
   <si>
-    <t>isues</t>
-  </si>
-  <si>
     <t>issues.reason</t>
   </si>
   <si>
@@ -1235,6 +1232,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Name of the company holding the existing policy/contract to be replaced.</t>
+  </si>
+  <si>
+    <t>Date on which issue resolution is due.</t>
   </si>
 </sst>
 </file>
@@ -1854,20 +1854,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0546D2BE-EB00-4D61-9BDC-7DB2C0656A13}">
   <dimension ref="A1:R213"/>
-  <sheetFormatPr defaultColWidth="84.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="84.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="37" style="3" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="35.5703125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" style="3" customWidth="1"/>
     <col min="6" max="16" width="10" style="3" customWidth="1"/>
-    <col min="17" max="17" width="36.33203125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="49.44140625" style="3" customWidth="1"/>
-    <col min="19" max="16384" width="84.33203125" style="3"/>
+    <col min="17" max="17" width="36.28515625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="49.42578125" style="3" customWidth="1"/>
+    <col min="19" max="16384" width="84.28515625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="33" t="s">
         <v>3</v>
       </c>
@@ -1886,7 +1886,7 @@
       <c r="N1" s="16"/>
       <c r="Q1" s="16"/>
     </row>
-    <row r="2" spans="1:18" s="5" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" s="5" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -1903,7 +1903,7 @@
       <c r="N2" s="15"/>
       <c r="Q2" s="15"/>
     </row>
-    <row r="3" spans="1:18" s="18" customFormat="1" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" s="18" customFormat="1" ht="158.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>4</v>
       </c>
@@ -1914,10 +1914,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="E3" s="29" t="s">
         <v>349</v>
-      </c>
-      <c r="E3" s="29" t="s">
-        <v>350</v>
       </c>
       <c r="F3" s="29" t="s">
         <v>7</v>
@@ -1941,7 +1941,7 @@
         <v>13</v>
       </c>
       <c r="M3" s="29" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="N3" s="29" t="s">
         <v>14</v>
@@ -1959,7 +1959,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
         <v>19</v>
       </c>
@@ -1981,7 +1981,7 @@
       <c r="Q4" s="36"/>
       <c r="R4" s="36"/>
     </row>
-    <row r="5" spans="1:18" ht="200.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="200.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>22</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>23</v>
@@ -2033,7 +2033,7 @@
       <c r="Q5" s="22"/>
       <c r="R5" s="4"/>
     </row>
-    <row r="6" spans="1:18" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>24</v>
       </c>
@@ -2085,7 +2085,7 @@
       <c r="Q6" s="22"/>
       <c r="R6" s="4"/>
     </row>
-    <row r="7" spans="1:18" ht="110.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -2191,7 +2191,7 @@
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
     </row>
-    <row r="9" spans="1:18" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -2243,7 +2243,7 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
     </row>
-    <row r="10" spans="1:18" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>40</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="171" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="171" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>50</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>56</v>
       </c>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="R13" s="2"/>
     </row>
-    <row r="14" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="R14" s="2"/>
     </row>
-    <row r="15" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>63</v>
       </c>
@@ -2565,7 +2565,7 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
     </row>
-    <row r="16" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>71</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>74</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>76</v>
       </c>
@@ -2779,7 +2779,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:18" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>81</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="21" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>85</v>
       </c>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="R21" s="2"/>
     </row>
-    <row r="22" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>88</v>
       </c>
@@ -2936,7 +2936,7 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
     </row>
-    <row r="23" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>90</v>
       </c>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="R23" s="2"/>
     </row>
-    <row r="24" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>92</v>
       </c>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="R24" s="2"/>
     </row>
-    <row r="25" spans="1:18" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>94</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:18" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>99</v>
       </c>
@@ -3154,7 +3154,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:18" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>102</v>
       </c>
@@ -3210,7 +3210,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:18" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>104</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:18" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>109</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>113</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="Q30" s="2"/>
       <c r="R30" s="8"/>
     </row>
-    <row r="31" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>115</v>
       </c>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="R31" s="8"/>
     </row>
-    <row r="32" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>118</v>
       </c>
@@ -3474,7 +3474,7 @@
       <c r="Q32" s="2"/>
       <c r="R32" s="8"/>
     </row>
-    <row r="33" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>120</v>
       </c>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="R33" s="8"/>
     </row>
-    <row r="34" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>122</v>
       </c>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="R34" s="8"/>
     </row>
-    <row r="35" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>125</v>
       </c>
@@ -3634,7 +3634,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="36" spans="1:18" s="10" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" s="10" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>128</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>132</v>
       </c>
@@ -3740,7 +3740,7 @@
       <c r="Q37" s="2"/>
       <c r="R37" s="27"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>134</v>
       </c>
@@ -3792,7 +3792,7 @@
       <c r="Q38" s="2"/>
       <c r="R38" s="27"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>137</v>
       </c>
@@ -3842,7 +3842,7 @@
       <c r="Q39" s="2"/>
       <c r="R39" s="27"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>139</v>
       </c>
@@ -3892,7 +3892,7 @@
       <c r="Q40" s="2"/>
       <c r="R40" s="27"/>
     </row>
-    <row r="41" spans="1:18" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>141</v>
       </c>
@@ -3940,10 +3940,10 @@
         <v>53</v>
       </c>
       <c r="R41" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>143</v>
       </c>
@@ -3994,10 +3994,10 @@
       </c>
       <c r="Q42" s="2"/>
       <c r="R42" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="43" spans="1:18" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>146</v>
       </c>
@@ -4047,7 +4047,7 @@
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>149</v>
       </c>
@@ -4099,7 +4099,7 @@
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>152</v>
       </c>
@@ -4151,7 +4151,7 @@
       <c r="Q45" s="2"/>
       <c r="R45" s="2"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>154</v>
       </c>
@@ -4203,7 +4203,7 @@
       <c r="Q46" s="2"/>
       <c r="R46" s="2"/>
     </row>
-    <row r="47" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>156</v>
       </c>
@@ -4255,7 +4255,7 @@
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>158</v>
       </c>
@@ -4307,7 +4307,7 @@
       <c r="Q48" s="2"/>
       <c r="R48" s="13"/>
     </row>
-    <row r="49" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>160</v>
       </c>
@@ -4361,7 +4361,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>163</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>167</v>
       </c>
@@ -4469,7 +4469,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>169</v>
       </c>
@@ -4523,7 +4523,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="34" t="s">
         <v>172</v>
       </c>
@@ -4545,7 +4545,7 @@
       <c r="Q53" s="35"/>
       <c r="R53" s="35"/>
     </row>
-    <row r="54" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>63</v>
       </c>
@@ -4597,7 +4597,7 @@
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>141</v>
       </c>
@@ -4647,7 +4647,7 @@
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>176</v>
       </c>
@@ -4699,7 +4699,7 @@
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
     </row>
-    <row r="57" spans="1:18" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>178</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>181</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="53.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>184</v>
       </c>
@@ -4855,11 +4855,11 @@
         <v>53</v>
       </c>
       <c r="Q59" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R59" s="2"/>
     </row>
-    <row r="60" spans="1:18" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" ht="216" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>186</v>
       </c>
@@ -4909,11 +4909,11 @@
         <v>53</v>
       </c>
       <c r="Q60" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R60" s="28"/>
     </row>
-    <row r="61" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>189</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>191</v>
       </c>
@@ -5017,13 +5017,13 @@
         <v>53</v>
       </c>
       <c r="Q62" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R62" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>193</v>
       </c>
@@ -5073,13 +5073,13 @@
         <v>53</v>
       </c>
       <c r="Q63" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R63" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>195</v>
       </c>
@@ -5087,7 +5087,7 @@
         <v>21</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>196</v>
@@ -5129,13 +5129,13 @@
         <v>53</v>
       </c>
       <c r="Q64" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R64" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:18" ht="24" x14ac:dyDescent="0.25">
       <c r="A65" s="34" t="s">
         <v>1</v>
       </c>
@@ -5157,7 +5157,7 @@
       <c r="Q65" s="35"/>
       <c r="R65" s="35"/>
     </row>
-    <row r="66" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>63</v>
       </c>
@@ -5209,7 +5209,7 @@
       <c r="Q66" s="2"/>
       <c r="R66" s="2"/>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>141</v>
       </c>
@@ -5259,7 +5259,7 @@
       <c r="Q67" s="2"/>
       <c r="R67" s="2"/>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>176</v>
       </c>
@@ -5311,7 +5311,7 @@
       <c r="Q68" s="2"/>
       <c r="R68" s="2"/>
     </row>
-    <row r="69" spans="1:18" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>178</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>203</v>
       </c>
@@ -5417,11 +5417,11 @@
         <v>53</v>
       </c>
       <c r="Q70" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R70" s="2"/>
     </row>
-    <row r="71" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>181</v>
       </c>
@@ -5475,7 +5475,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>209</v>
       </c>
@@ -5529,7 +5529,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>212</v>
       </c>
@@ -5579,7 +5579,7 @@
       <c r="Q73" s="2"/>
       <c r="R73" s="2"/>
     </row>
-    <row r="74" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="34" t="s">
         <v>214</v>
       </c>
@@ -5601,7 +5601,7 @@
       <c r="Q74" s="35"/>
       <c r="R74" s="35"/>
     </row>
-    <row r="75" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>63</v>
       </c>
@@ -5653,7 +5653,7 @@
       <c r="Q75" s="2"/>
       <c r="R75" s="2"/>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>141</v>
       </c>
@@ -5703,7 +5703,7 @@
       <c r="Q76" s="2"/>
       <c r="R76" s="2"/>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>176</v>
       </c>
@@ -5755,7 +5755,7 @@
       <c r="Q77" s="2"/>
       <c r="R77" s="2"/>
     </row>
-    <row r="78" spans="1:18" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:18" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>178</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>181</v>
       </c>
@@ -5863,9 +5863,9 @@
         <v>217</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>218</v>
+        <v>184</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>77</v>
@@ -5911,13 +5911,13 @@
         <v>53</v>
       </c>
       <c r="Q80" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="R80" s="2"/>
     </row>
-    <row r="81" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>21</v>
@@ -5926,61 +5926,61 @@
         <v>204</v>
       </c>
       <c r="D81" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="E81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="N81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O81" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P81" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q81" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="R81" s="2"/>
+    </row>
+    <row r="82" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="E81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I81" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="K81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="N81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O81" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P81" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q81" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="R81" s="2"/>
-    </row>
-    <row r="82" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A82" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C82" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D82" s="6" t="s">
         <v>222</v>
-      </c>
-      <c r="D82" s="6" t="s">
-        <v>223</v>
       </c>
       <c r="E82" s="9" t="s">
         <v>53</v>
@@ -6019,24 +6019,24 @@
         <v>53</v>
       </c>
       <c r="Q82" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="R82" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="R82" s="14" t="s">
+    </row>
+    <row r="83" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
         <v>225</v>
-      </c>
-    </row>
-    <row r="83" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A83" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C83" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D83" s="6" t="s">
         <v>227</v>
-      </c>
-      <c r="D83" s="6" t="s">
-        <v>228</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>53</v>
@@ -6075,21 +6075,21 @@
         <v>53</v>
       </c>
       <c r="Q83" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="R83" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="R83" s="14" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>210</v>
+        <v>354</v>
       </c>
       <c r="D84" s="20" t="s">
         <v>69</v>
@@ -6132,10 +6132,10 @@
       </c>
       <c r="Q84" s="2"/>
       <c r="R84" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="85" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>189</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:18" ht="24" x14ac:dyDescent="0.25">
       <c r="A86" s="34" t="s">
         <v>2</v>
       </c>
@@ -6211,7 +6211,7 @@
       <c r="Q86" s="35"/>
       <c r="R86" s="35"/>
     </row>
-    <row r="87" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>63</v>
       </c>
@@ -6219,7 +6219,7 @@
         <v>21</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>174</v>
@@ -6263,7 +6263,7 @@
       <c r="Q87" s="2"/>
       <c r="R87" s="2"/>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>141</v>
       </c>
@@ -6313,7 +6313,7 @@
       <c r="Q88" s="2"/>
       <c r="R88" s="2"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>176</v>
       </c>
@@ -6348,7 +6348,7 @@
         <v>23</v>
       </c>
       <c r="L89" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M89" s="2" t="s">
         <v>23</v>
@@ -6365,7 +6365,7 @@
       <c r="Q89" s="2"/>
       <c r="R89" s="2"/>
     </row>
-    <row r="90" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>178</v>
       </c>
@@ -6415,11 +6415,11 @@
         <v>53</v>
       </c>
       <c r="Q90" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R90" s="2"/>
     </row>
-    <row r="91" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>181</v>
       </c>
@@ -6473,15 +6473,15 @@
         <v>217</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>77</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D92" s="6"/>
       <c r="E92" s="9" t="s">
@@ -6523,15 +6523,15 @@
       <c r="Q92" s="2"/>
       <c r="R92" s="2"/>
     </row>
-    <row r="93" spans="1:18" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:18" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>26</v>
@@ -6575,18 +6575,18 @@
       <c r="Q93" s="4"/>
       <c r="R93" s="4"/>
     </row>
-    <row r="94" spans="1:18" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C94" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D94" s="6" t="s">
         <v>239</v>
-      </c>
-      <c r="D94" s="6" t="s">
-        <v>240</v>
       </c>
       <c r="E94" s="9" t="s">
         <v>53</v>
@@ -6627,18 +6627,18 @@
       <c r="Q94" s="2"/>
       <c r="R94" s="2"/>
     </row>
-    <row r="95" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C95" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D95" s="6" t="s">
         <v>242</v>
-      </c>
-      <c r="D95" s="6" t="s">
-        <v>243</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>53</v>
@@ -6679,9 +6679,9 @@
       <c r="Q95" s="2"/>
       <c r="R95" s="2"/>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>41</v>
@@ -6729,15 +6729,15 @@
       <c r="Q96" s="2"/>
       <c r="R96" s="2"/>
     </row>
-    <row r="97" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>147</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="9" t="s">
@@ -6777,19 +6777,19 @@
         <v>53</v>
       </c>
       <c r="Q97" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="R97" s="2"/>
+    </row>
+    <row r="98" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="R97" s="2"/>
-    </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A98" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>147</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D98" s="6"/>
       <c r="E98" s="9" t="s">
@@ -6831,15 +6831,15 @@
       <c r="Q98" s="2"/>
       <c r="R98" s="2"/>
     </row>
-    <row r="99" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D99" s="20" t="s">
         <v>69</v>
@@ -6883,18 +6883,18 @@
       <c r="Q99" s="2"/>
       <c r="R99" s="2"/>
     </row>
-    <row r="100" spans="1:18" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:18" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C100" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D100" s="6" t="s">
         <v>253</v>
-      </c>
-      <c r="D100" s="6" t="s">
-        <v>254</v>
       </c>
       <c r="E100" s="9" t="s">
         <v>53</v>
@@ -6935,9 +6935,9 @@
       <c r="Q100" s="2"/>
       <c r="R100" s="2"/>
     </row>
-    <row r="101" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>21</v>
@@ -6946,7 +6946,7 @@
         <v>204</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>53</v>
@@ -6985,19 +6985,19 @@
         <v>53</v>
       </c>
       <c r="Q101" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="R101" s="2"/>
+    </row>
+    <row r="102" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="R101" s="2"/>
-    </row>
-    <row r="102" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A102" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D102" s="20" t="s">
         <v>69</v>
@@ -7041,9 +7041,9 @@
       <c r="Q102" s="2"/>
       <c r="R102" s="2"/>
     </row>
-    <row r="103" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>21</v>
@@ -7092,21 +7092,21 @@
       </c>
       <c r="Q103" s="2"/>
       <c r="R103" s="14" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="104" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
         <v>261</v>
-      </c>
-    </row>
-    <row r="104" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A104" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E104" s="9" t="s">
         <v>53</v>
@@ -7145,19 +7145,19 @@
         <v>53</v>
       </c>
       <c r="Q104" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R104" s="14"/>
     </row>
-    <row r="105" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C105" s="14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D105" s="6"/>
       <c r="E105" s="9" t="s">
@@ -7197,19 +7197,19 @@
         <v>53</v>
       </c>
       <c r="Q105" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R105" s="14"/>
     </row>
-    <row r="106" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C106" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D106" s="20" t="s">
         <v>69</v>
@@ -7251,19 +7251,19 @@
         <v>53</v>
       </c>
       <c r="Q106" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R106" s="14"/>
     </row>
-    <row r="107" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:18" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C107" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>69</v>
@@ -7307,9 +7307,9 @@
       <c r="Q107" s="2"/>
       <c r="R107" s="14"/>
     </row>
-    <row r="108" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>21</v>
@@ -7358,21 +7358,21 @@
       </c>
       <c r="Q108" s="2"/>
       <c r="R108" s="14" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="109" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="109" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C109" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D109" s="6" t="s">
         <v>272</v>
-      </c>
-      <c r="D109" s="6" t="s">
-        <v>273</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>53</v>
@@ -7411,13 +7411,13 @@
         <v>53</v>
       </c>
       <c r="Q109" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R109" s="14"/>
+    </row>
+    <row r="110" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="22" t="s">
         <v>274</v>
-      </c>
-      <c r="R109" s="14"/>
-    </row>
-    <row r="110" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="22" t="s">
-        <v>275</v>
       </c>
       <c r="B110" s="22"/>
       <c r="C110" s="22"/>
@@ -7453,65 +7453,65 @@
         <v>53</v>
       </c>
       <c r="Q110" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R110" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="111" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="2" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="111" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C111" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D111" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="D111" s="6" t="s">
+      <c r="E111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O111" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P111" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q111" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R111" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="112" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="E111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O111" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P111" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q111" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R111" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="112" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>21</v>
@@ -7553,15 +7553,15 @@
         <v>53</v>
       </c>
       <c r="Q112" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R112" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="113" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="113" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>21</v>
@@ -7601,15 +7601,15 @@
         <v>53</v>
       </c>
       <c r="Q113" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R113" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="114" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="114" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>21</v>
@@ -7651,15 +7651,15 @@
         <v>53</v>
       </c>
       <c r="Q114" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R114" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="115" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="115" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>21</v>
@@ -7701,15 +7701,15 @@
         <v>53</v>
       </c>
       <c r="Q115" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R115" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="116" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="116" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>21</v>
@@ -7751,15 +7751,15 @@
         <v>53</v>
       </c>
       <c r="Q116" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R116" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="117" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="117" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>21</v>
@@ -7801,15 +7801,15 @@
         <v>53</v>
       </c>
       <c r="Q117" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R117" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="118" spans="1:18" ht="105" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="118" spans="1:18" ht="105" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>105</v>
@@ -7818,48 +7818,48 @@
         <v>106</v>
       </c>
       <c r="D118" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O118" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P118" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q118" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R118" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="119" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="22" t="s">
         <v>287</v>
-      </c>
-      <c r="E118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O118" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P118" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q118" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R118" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="119" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="22" t="s">
-        <v>288</v>
       </c>
       <c r="B119" s="22"/>
       <c r="C119" s="22"/>
@@ -7895,65 +7895,65 @@
         <v>53</v>
       </c>
       <c r="Q119" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R119" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="120" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="2" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="120" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D120" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="E120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O120" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P120" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q120" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R120" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="121" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="E120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O120" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P120" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q120" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R120" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="121" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>21</v>
@@ -7995,15 +7995,15 @@
         <v>53</v>
       </c>
       <c r="Q121" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R121" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="122" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="122" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>21</v>
@@ -8045,15 +8045,15 @@
         <v>53</v>
       </c>
       <c r="Q122" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R122" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="123" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="123" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>21</v>
@@ -8095,15 +8095,15 @@
         <v>53</v>
       </c>
       <c r="Q123" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R123" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="124" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="124" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>21</v>
@@ -8145,15 +8145,15 @@
         <v>53</v>
       </c>
       <c r="Q124" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R124" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="125" spans="1:18" ht="135" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="125" spans="1:18" ht="135" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>105</v>
@@ -8162,48 +8162,48 @@
         <v>106</v>
       </c>
       <c r="D125" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="E125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O125" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P125" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q125" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R125" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="126" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="22" t="s">
         <v>291</v>
-      </c>
-      <c r="E125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O125" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P125" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q125" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R125" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="126" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="22" t="s">
-        <v>292</v>
       </c>
       <c r="B126" s="22"/>
       <c r="C126" s="22"/>
@@ -8239,15 +8239,15 @@
         <v>53</v>
       </c>
       <c r="Q126" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R126" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="127" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="127" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>21</v>
@@ -8256,48 +8256,48 @@
         <v>114</v>
       </c>
       <c r="D127" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O127" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P127" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q127" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R127" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="128" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="E127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O127" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P127" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q127" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R127" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="128" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>21</v>
@@ -8339,15 +8339,15 @@
         <v>53</v>
       </c>
       <c r="Q128" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R128" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="129" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="129" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>21</v>
@@ -8387,15 +8387,15 @@
         <v>53</v>
       </c>
       <c r="Q129" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R129" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="130" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="130" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>21</v>
@@ -8437,15 +8437,15 @@
         <v>53</v>
       </c>
       <c r="Q130" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R130" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="131" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="131" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>21</v>
@@ -8485,15 +8485,15 @@
         <v>53</v>
       </c>
       <c r="Q131" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R131" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="132" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="132" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>21</v>
@@ -8535,15 +8535,15 @@
         <v>53</v>
       </c>
       <c r="Q132" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R132" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="133" spans="1:18" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="133" spans="1:18" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>105</v>
@@ -8552,48 +8552,48 @@
         <v>129</v>
       </c>
       <c r="D133" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="E133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O133" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P133" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q133" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R133" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="134" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="22" t="s">
         <v>293</v>
-      </c>
-      <c r="E133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O133" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P133" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q133" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R133" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="134" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="22" t="s">
-        <v>294</v>
       </c>
       <c r="B134" s="22"/>
       <c r="C134" s="22"/>
@@ -8629,15 +8629,15 @@
         <v>53</v>
       </c>
       <c r="Q134" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R134" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="135" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="135" spans="1:18" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>21</v>
@@ -8646,48 +8646,48 @@
         <v>114</v>
       </c>
       <c r="D135" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="E135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O135" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P135" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q135" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R135" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="136" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="E135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O135" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P135" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q135" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R135" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="136" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>21</v>
@@ -8727,15 +8727,15 @@
         <v>53</v>
       </c>
       <c r="Q136" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R136" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="137" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="137" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>21</v>
@@ -8777,15 +8777,15 @@
         <v>53</v>
       </c>
       <c r="Q137" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R137" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="138" spans="1:18" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="138" spans="1:18" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>105</v>
@@ -8794,7 +8794,7 @@
         <v>129</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E138" s="9" t="s">
         <v>53</v>
@@ -8827,15 +8827,15 @@
         <v>53</v>
       </c>
       <c r="Q138" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R138" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="139" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="139" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="22" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B139" s="22"/>
       <c r="C139" s="22"/>
@@ -8871,21 +8871,21 @@
         <v>53</v>
       </c>
       <c r="Q139" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R139" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="140" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="140" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D140" s="6"/>
       <c r="E140" s="9" t="s">
@@ -8919,13 +8919,13 @@
         <v>53</v>
       </c>
       <c r="Q140" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R140" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="141" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="141" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>27</v>
       </c>
@@ -8969,13 +8969,13 @@
         <v>53</v>
       </c>
       <c r="Q141" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R141" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="142" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="142" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>33</v>
       </c>
@@ -9017,13 +9017,13 @@
         <v>53</v>
       </c>
       <c r="Q142" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R142" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="143" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="143" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>37</v>
       </c>
@@ -9067,13 +9067,13 @@
         <v>53</v>
       </c>
       <c r="Q143" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R143" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="144" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="144" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>40</v>
       </c>
@@ -9115,13 +9115,13 @@
         <v>53</v>
       </c>
       <c r="Q144" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R144" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="145" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="145" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>45</v>
       </c>
@@ -9165,13 +9165,13 @@
         <v>53</v>
       </c>
       <c r="Q145" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R145" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="146" spans="1:18" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="146" spans="1:18" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>50</v>
       </c>
@@ -9215,13 +9215,13 @@
         <v>53</v>
       </c>
       <c r="Q146" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R146" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="147" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="147" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>56</v>
       </c>
@@ -9265,13 +9265,13 @@
         <v>53</v>
       </c>
       <c r="Q147" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R147" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="148" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="148" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>60</v>
       </c>
@@ -9313,13 +9313,13 @@
         <v>53</v>
       </c>
       <c r="Q148" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R148" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="149" spans="1:18" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="149" spans="1:18" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>63</v>
       </c>
@@ -9363,13 +9363,13 @@
         <v>53</v>
       </c>
       <c r="Q149" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R149" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="150" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="150" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>66</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>67</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D150" s="20" t="s">
         <v>69</v>
@@ -9413,13 +9413,13 @@
         <v>53</v>
       </c>
       <c r="Q150" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R150" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="151" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="151" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>71</v>
       </c>
@@ -9427,7 +9427,7 @@
         <v>21</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D151" s="6" t="s">
         <v>73</v>
@@ -9463,13 +9463,13 @@
         <v>53</v>
       </c>
       <c r="Q151" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R151" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="152" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="152" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>74</v>
       </c>
@@ -9477,7 +9477,7 @@
         <v>21</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D152" s="6"/>
       <c r="E152" s="9" t="s">
@@ -9511,13 +9511,13 @@
         <v>53</v>
       </c>
       <c r="Q152" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R152" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="153" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="153" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>76</v>
       </c>
@@ -9561,13 +9561,13 @@
         <v>53</v>
       </c>
       <c r="Q153" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R153" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="154" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="154" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>81</v>
       </c>
@@ -9612,13 +9612,13 @@
         <v>53</v>
       </c>
       <c r="Q154" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R154" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="155" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="155" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>85</v>
       </c>
@@ -9663,13 +9663,13 @@
         <v>53</v>
       </c>
       <c r="Q155" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R155" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="156" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="156" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>88</v>
       </c>
@@ -9712,13 +9712,13 @@
         <v>53</v>
       </c>
       <c r="Q156" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R156" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="157" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="157" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>90</v>
       </c>
@@ -9763,13 +9763,13 @@
         <v>53</v>
       </c>
       <c r="Q157" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R157" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="158" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="158" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>92</v>
       </c>
@@ -9812,13 +9812,13 @@
         <v>53</v>
       </c>
       <c r="Q158" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R158" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="159" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="159" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>94</v>
       </c>
@@ -9863,13 +9863,13 @@
         <v>53</v>
       </c>
       <c r="Q159" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R159" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="160" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="160" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>99</v>
       </c>
@@ -9914,13 +9914,13 @@
         <v>53</v>
       </c>
       <c r="Q160" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R160" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="161" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="161" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>102</v>
       </c>
@@ -9965,13 +9965,13 @@
         <v>53</v>
       </c>
       <c r="Q161" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R161" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="162" spans="1:18" s="10" customFormat="1" ht="240" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="162" spans="1:18" s="10" customFormat="1" ht="240" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>104</v>
       </c>
@@ -9982,7 +9982,7 @@
         <v>106</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E162" s="9" t="s">
         <v>53</v>
@@ -10016,13 +10016,13 @@
         <v>53</v>
       </c>
       <c r="Q162" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R162" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="163" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="163" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>109</v>
       </c>
@@ -10033,7 +10033,7 @@
         <v>110</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E163" s="9" t="s">
         <v>53</v>
@@ -10066,13 +10066,13 @@
         <v>53</v>
       </c>
       <c r="Q163" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R163" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="164" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="164" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>113</v>
       </c>
@@ -10117,13 +10117,13 @@
         <v>53</v>
       </c>
       <c r="Q164" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R164" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="165" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="165" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>115</v>
       </c>
@@ -10168,13 +10168,13 @@
         <v>53</v>
       </c>
       <c r="Q165" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R165" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="166" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="166" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>118</v>
       </c>
@@ -10217,13 +10217,13 @@
         <v>53</v>
       </c>
       <c r="Q166" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R166" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="167" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="167" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>120</v>
       </c>
@@ -10268,13 +10268,13 @@
         <v>53</v>
       </c>
       <c r="Q167" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R167" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="168" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="168" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>122</v>
       </c>
@@ -10317,13 +10317,13 @@
         <v>53</v>
       </c>
       <c r="Q168" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R168" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="169" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="169" spans="1:18" s="10" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>125</v>
       </c>
@@ -10368,13 +10368,13 @@
         <v>53</v>
       </c>
       <c r="Q169" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R169" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="170" spans="1:18" s="10" customFormat="1" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="170" spans="1:18" s="10" customFormat="1" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>128</v>
       </c>
@@ -10385,7 +10385,7 @@
         <v>129</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E170" s="9" t="s">
         <v>53</v>
@@ -10419,13 +10419,13 @@
         <v>53</v>
       </c>
       <c r="Q170" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R170" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="171" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="171" spans="1:18" s="10" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>132</v>
       </c>
@@ -10470,13 +10470,13 @@
         <v>53</v>
       </c>
       <c r="Q171" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R171" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="172" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="172" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>134</v>
       </c>
@@ -10520,13 +10520,13 @@
         <v>53</v>
       </c>
       <c r="Q172" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R172" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="173" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="173" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>137</v>
       </c>
@@ -10568,13 +10568,13 @@
         <v>53</v>
       </c>
       <c r="Q173" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R173" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="174" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="174" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>139</v>
       </c>
@@ -10616,13 +10616,13 @@
         <v>53</v>
       </c>
       <c r="Q174" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R174" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="175" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="175" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>141</v>
       </c>
@@ -10664,13 +10664,13 @@
         <v>53</v>
       </c>
       <c r="Q175" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R175" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="176" spans="1:18" ht="135" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="176" spans="1:18" ht="135" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>143</v>
       </c>
@@ -10714,13 +10714,13 @@
         <v>53</v>
       </c>
       <c r="Q176" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R176" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="177" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="177" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>149</v>
       </c>
@@ -10764,13 +10764,13 @@
         <v>53</v>
       </c>
       <c r="Q177" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R177" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="178" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="178" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>152</v>
       </c>
@@ -10814,13 +10814,13 @@
         <v>53</v>
       </c>
       <c r="Q178" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R178" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="179" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="179" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>154</v>
       </c>
@@ -10864,13 +10864,13 @@
         <v>53</v>
       </c>
       <c r="Q179" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R179" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="180" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="180" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>156</v>
       </c>
@@ -10878,7 +10878,7 @@
         <v>150</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D180" s="20" t="s">
         <v>69</v>
@@ -10914,13 +10914,13 @@
         <v>53</v>
       </c>
       <c r="Q180" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R180" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="181" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="181" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>158</v>
       </c>
@@ -10928,7 +10928,7 @@
         <v>150</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D181" s="20" t="s">
         <v>69</v>
@@ -10964,13 +10964,13 @@
         <v>53</v>
       </c>
       <c r="Q181" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R181" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="182" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="182" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>160</v>
       </c>
@@ -10978,7 +10978,7 @@
         <v>150</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D182" s="20" t="s">
         <v>69</v>
@@ -11014,13 +11014,13 @@
         <v>53</v>
       </c>
       <c r="Q182" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R182" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="183" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="183" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>163</v>
       </c>
@@ -11064,13 +11064,13 @@
         <v>53</v>
       </c>
       <c r="Q183" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R183" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="184" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="184" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>167</v>
       </c>
@@ -11114,13 +11114,13 @@
         <v>53</v>
       </c>
       <c r="Q184" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R184" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="185" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="185" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>169</v>
       </c>
@@ -11164,215 +11164,215 @@
         <v>53</v>
       </c>
       <c r="Q185" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R185" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="186" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="186" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C186" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D186" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D186" s="6" t="s">
+      <c r="E186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O186" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P186" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q186" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R186" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="187" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="E186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O186" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P186" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q186" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R186" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="187" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="2" t="s">
+      <c r="B187" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B187" s="2" t="s">
+      <c r="C187" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="C187" s="2" t="s">
+      <c r="D187" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="D187" s="6" t="s">
+      <c r="E187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O187" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P187" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q187" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R187" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="188" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
         <v>313</v>
-      </c>
-      <c r="E187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O187" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P187" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q187" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R187" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="188" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="2" t="s">
-        <v>314</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C188" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D188" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="D188" s="6" t="s">
+      <c r="E188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O188" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P188" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q188" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R188" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="189" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="E188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O188" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P188" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q188" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R188" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="189" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="2" t="s">
-        <v>317</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C189" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D189" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="D189" s="6" t="s">
+      <c r="E189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O189" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P189" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q189" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R189" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="190" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="22" t="s">
         <v>319</v>
-      </c>
-      <c r="E189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O189" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P189" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q189" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R189" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="190" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="22" t="s">
-        <v>320</v>
       </c>
       <c r="B190" s="22"/>
       <c r="C190" s="22"/>
@@ -11408,13 +11408,13 @@
         <v>53</v>
       </c>
       <c r="Q190" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R190" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="191" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="191" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>27</v>
       </c>
@@ -11425,7 +11425,7 @@
         <v>28</v>
       </c>
       <c r="D191" s="6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>53</v>
@@ -11458,13 +11458,13 @@
         <v>53</v>
       </c>
       <c r="Q191" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R191" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="192" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="192" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>33</v>
       </c>
@@ -11508,13 +11508,13 @@
         <v>53</v>
       </c>
       <c r="Q192" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R192" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="193" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="193" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>50</v>
       </c>
@@ -11555,22 +11555,22 @@
         <v>53</v>
       </c>
       <c r="Q193" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R193" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="194" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="194" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C194" s="2"/>
       <c r="D194" s="6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E194" s="9" t="s">
         <v>53</v>
@@ -11603,15 +11603,15 @@
         <v>53</v>
       </c>
       <c r="Q194" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R194" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="195" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="195" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>21</v>
@@ -11653,15 +11653,15 @@
         <v>53</v>
       </c>
       <c r="Q195" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R195" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="196" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="196" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>21</v>
@@ -11703,15 +11703,15 @@
         <v>53</v>
       </c>
       <c r="Q196" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R196" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="197" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="197" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>21</v>
@@ -11753,15 +11753,15 @@
         <v>53</v>
       </c>
       <c r="Q197" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R197" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="198" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="198" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>21</v>
@@ -11801,21 +11801,21 @@
         <v>53</v>
       </c>
       <c r="Q198" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R198" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="199" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="199" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D199" s="6" t="s">
         <v>47</v>
@@ -11851,65 +11851,65 @@
         <v>53</v>
       </c>
       <c r="Q199" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R199" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="200" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="200" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B200" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="B200" s="2" t="s">
+      <c r="C200" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C200" s="2" t="s">
+      <c r="D200" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="D200" s="6" t="s">
+      <c r="E200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O200" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P200" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q200" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R200" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="201" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="22" t="s">
         <v>329</v>
-      </c>
-      <c r="E200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O200" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P200" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q200" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R200" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="201" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="22" t="s">
-        <v>330</v>
       </c>
       <c r="B201" s="22"/>
       <c r="C201" s="22"/>
@@ -11945,21 +11945,21 @@
         <v>53</v>
       </c>
       <c r="Q201" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R201" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="202" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="202" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D202" s="6"/>
       <c r="E202" s="9" t="s">
@@ -11993,21 +11993,21 @@
         <v>53</v>
       </c>
       <c r="Q202" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R202" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="203" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="203" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C203" s="2" t="s">
         <v>331</v>
-      </c>
-      <c r="B203" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>332</v>
       </c>
       <c r="D203" s="6"/>
       <c r="E203" s="9" t="s">
@@ -12041,21 +12041,21 @@
         <v>53</v>
       </c>
       <c r="Q203" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R203" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="204" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="204" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C204" s="3" t="s">
         <v>333</v>
-      </c>
-      <c r="B204" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C204" s="3" t="s">
-        <v>334</v>
       </c>
       <c r="D204" s="6"/>
       <c r="E204" s="9" t="s">
@@ -12089,21 +12089,21 @@
         <v>53</v>
       </c>
       <c r="Q204" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R204" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="205" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="205" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C205" s="2" t="s">
         <v>335</v>
-      </c>
-      <c r="B205" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C205" s="2" t="s">
-        <v>336</v>
       </c>
       <c r="D205" s="6"/>
       <c r="E205" s="9" t="s">
@@ -12137,63 +12137,63 @@
         <v>53</v>
       </c>
       <c r="Q205" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R205" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="206" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="206" spans="1:18" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>77</v>
       </c>
       <c r="C206" s="2"/>
       <c r="D206" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O206" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P206" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q206" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R206" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="207" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="22" t="s">
         <v>338</v>
-      </c>
-      <c r="E206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O206" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P206" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q206" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R206" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="207" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A207" s="22" t="s">
-        <v>339</v>
       </c>
       <c r="B207" s="22"/>
       <c r="C207" s="22"/>
@@ -12229,21 +12229,21 @@
         <v>53</v>
       </c>
       <c r="Q207" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R207" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="208" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="208" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C208" s="2" t="s">
         <v>331</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>332</v>
       </c>
       <c r="D208" s="6"/>
       <c r="E208" s="9" t="s">
@@ -12277,21 +12277,21 @@
         <v>53</v>
       </c>
       <c r="Q208" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R208" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="209" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="209" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C209" s="3" t="s">
         <v>333</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C209" s="3" t="s">
-        <v>334</v>
       </c>
       <c r="D209" s="6"/>
       <c r="E209" s="9" t="s">
@@ -12325,21 +12325,21 @@
         <v>53</v>
       </c>
       <c r="Q209" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R209" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="210" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="210" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C210" s="2" t="s">
         <v>335</v>
-      </c>
-      <c r="B210" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C210" s="2" t="s">
-        <v>336</v>
       </c>
       <c r="D210" s="6"/>
       <c r="E210" s="9" t="s">
@@ -12373,110 +12373,110 @@
         <v>53</v>
       </c>
       <c r="Q210" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R210" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="211" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="211" spans="1:18" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B211" s="2" t="s">
         <v>77</v>
       </c>
       <c r="C211" s="2"/>
       <c r="D211" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O211" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P211" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q211" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R211" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="212" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="O212" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P212" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q212" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R212" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="213" spans="1:18" ht="75" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="E211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O211" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P211" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q211" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R211" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="212" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="L212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="O212" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P212" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q212" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="R212" s="14" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="213" spans="1:18" ht="72" x14ac:dyDescent="0.3">
-      <c r="A213" s="2" t="s">
-        <v>342</v>
       </c>
       <c r="B213" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C213" s="14" t="s">
+        <v>342</v>
+      </c>
+      <c r="D213" s="6" t="s">
         <v>343</v>
-      </c>
-      <c r="D213" s="6" t="s">
-        <v>344</v>
       </c>
       <c r="E213" s="9" t="s">
         <v>53</v>
@@ -12515,7 +12515,7 @@
         <v>53</v>
       </c>
       <c r="Q213" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R213" s="14"/>
     </row>

</xml_diff>